<commit_message>
Fixed: if merchant and location is not parsed, do not take it from the rule.
</commit_message>
<xml_diff>
--- a/data/example/output/dataset.analysis.xlsx
+++ b/data/example/output/dataset.analysis.xlsx
@@ -175,41 +175,166 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Transaction Categories Overview</a:t>
+              <a:t>Income vs. Expenses</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
     </title>
     <plotArea>
-      <pieChart>
-        <varyColors val="1"/>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="stacked"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Summary'!F6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E7D32"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Summary'!$H$7:$H$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Summary'!$F$7:$F$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Summary'!G6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="A5D6A7"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Summary'!$H$7:$H$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Summary'!$G$7:$G$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Summary'!H6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="C62828"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Summary'!$H$7:$H$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Summary'!$H$7:$H$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
           <tx>
             <strRef>
               <f>'Summary'!I6</f>
             </strRef>
           </tx>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="EF9A9A"/>
+            </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Summary'!$H$7:$H$10</f>
+              <f>'Summary'!$H$7:$H$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$7:$I$10</f>
+              <f>'Summary'!$I$7:$I$8</f>
             </numRef>
           </val>
         </ser>
-        <firstSliceAng val="0"/>
-      </pieChart>
+        <gapWidth val="150"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Amount (CHF)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
     </plotArea>
     <legend>
       <legendPos val="r"/>
@@ -811,14 +936,29 @@
       </c>
     </row>
     <row r="6">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>refund (credit)</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Transaction Category</t>
+          <t>expenses</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Amount (CHF)</t>
+          <t>refund (debit)</t>
         </is>
       </c>
     </row>
@@ -838,13 +978,22 @@
           <t>Debit (CHF)</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
+      <c r="F7" s="5" t="n">
+        <v>11166.35</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>1888.95</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I7" s="5" t="n">
-        <v>11166.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -859,13 +1008,22 @@
       <c r="C8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>3104.36</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>3104.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -880,14 +1038,6 @@
       <c r="C9" s="5" t="n">
         <v>3104.36</v>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Refund</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="n">
-        <v>1888.95</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -900,14 +1050,6 @@
       </c>
       <c r="C10" s="5" t="n">
         <v>0</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Transfer</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>450</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
Replaced categorization as "Beispiel" with actual category and subcategory.
</commit_message>
<xml_diff>
--- a/data/example/output/dataset.analysis.xlsx
+++ b/data/example/output/dataset.analysis.xlsx
@@ -382,12 +382,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$8:$A$9</f>
+              <f>'Overviews by category'!$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$8:$B$9</f>
+              <f>'Overviews by category'!$B$8</f>
             </numRef>
           </val>
         </ser>
@@ -440,12 +440,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$30:$A$36</f>
+              <f>'Overviews by category'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$30:$B$36</f>
+              <f>'Overviews by category'!$B$30:$B$35</f>
             </numRef>
           </val>
         </ser>
@@ -1150,17 +1150,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Beispiel</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>4200</v>
+        <v>11166.35</v>
       </c>
     </row>
     <row r="27">
@@ -1239,17 +1229,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Beispiel</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="n">
-        <v>25</v>
+        <v>110</v>
       </c>
     </row>
     <row r="49">
@@ -1313,7 +1293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1663,17 +1643,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Beispiel</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
         <v>4200</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="D36" s="5" t="n">
-        <v>4175</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="37">
@@ -1690,6 +1670,22 @@
       </c>
       <c r="D37" s="5" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Finanzen</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>-25</v>
       </c>
     </row>
   </sheetData>
@@ -2286,12 +2282,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Beispiel</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Counterparty</t>
+          <t>Lohn</t>
         </is>
       </c>
       <c r="C43" s="5" t="n">
@@ -2307,12 +2303,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Beispiel</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Counterparty IBAN</t>
+          <t>Spenden</t>
         </is>
       </c>
       <c r="C44" s="5" t="n">

</xml_diff>